<commit_message>
Update  for new bar charts
</commit_message>
<xml_diff>
--- a/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/outputs_IAEE_2025_run_2021_utilization_share.xlsx
+++ b/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/outputs_IAEE_2025_run_2021_utilization_share.xlsx
@@ -453,14 +453,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>425972</v>
+        <v>87930</v>
       </c>
       <c r="C2" t="n">
-        <v>425972</v>
+        <v>87930</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -469,14 +469,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>154366</v>
+        <v>68390</v>
       </c>
       <c r="C3" t="n">
-        <v>154366</v>
+        <v>68390</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -485,46 +485,46 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>322409.9999999999</v>
+        <v>398886.1359907001</v>
       </c>
       <c r="C4" t="n">
-        <v>322410</v>
+        <v>587177</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9999999999999997</v>
+        <v>0.6793286112887598</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>39080</v>
+        <v>322409.9999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>39080</v>
+        <v>322410</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>0.9999999999999997</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87930</v>
+        <v>25402</v>
       </c>
       <c r="C6" t="n">
-        <v>87930</v>
+        <v>25402</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -533,30 +533,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>398886.1359907001</v>
+        <v>154366</v>
       </c>
       <c r="C7" t="n">
-        <v>587177</v>
+        <v>154366</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6793286112887598</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25402</v>
+        <v>39080</v>
       </c>
       <c r="C8" t="n">
-        <v>25402</v>
+        <v>39080</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -565,14 +565,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>469937</v>
+        <v>117240</v>
       </c>
       <c r="C9" t="n">
-        <v>469937</v>
+        <v>117240</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
@@ -613,14 +613,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>68390</v>
+        <v>425972</v>
       </c>
       <c r="C12" t="n">
-        <v>68390</v>
+        <v>425972</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -629,14 +629,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>117240</v>
+        <v>469937</v>
       </c>
       <c r="C13" t="n">
-        <v>117240</v>
+        <v>469937</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -671,7 +671,7 @@
         <v>1529982</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8688653202804499</v>
+        <v>0.8688653202804498</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add updated files of flowmaps
</commit_message>
<xml_diff>
--- a/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/outputs_IAEE_2025_run_2021_utilization_share.xlsx
+++ b/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/outputs_IAEE_2025_run_2021_utilization_share.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>